<commit_message>
Trying to fix odes problems
</commit_message>
<xml_diff>
--- a/data/processed/BR_processed_ind.xlsx
+++ b/data/processed/BR_processed_ind.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y67"/>
+  <dimension ref="A1:AA67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,40 +516,50 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
+          <t>qP_sqrt</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>rP_sqrt</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>Xlag1</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Plag1</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>X_calc</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>V_calc</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>mu_calc</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>dXdt_calc</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>dVdt_calc</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Xlag1_calc</t>
         </is>
@@ -614,28 +624,34 @@
         <v>0.03252295278732637</v>
       </c>
       <c r="R2" t="n">
+        <v>0.03754548692326653</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.1803412121156071</v>
+      </c>
+      <c r="T2" t="n">
         <v>19.55000000000009</v>
       </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" t="n">
-        <v>26.65401311124306</v>
-      </c>
       <c r="U2" t="n">
-        <v>1.848679151181504</v>
+        <v>0</v>
       </c>
       <c r="V2" t="n">
-        <v>0.2252313546719042</v>
+        <v>26.65401336848298</v>
       </c>
       <c r="W2" t="n">
-        <v>5.970158382675687</v>
+        <v>1.848679229473595</v>
       </c>
       <c r="X2" t="n">
+        <v>0.2252279510788963</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>5.970067722284991</v>
+      </c>
+      <c r="Z2" t="n">
         <v>0.0023</v>
       </c>
-      <c r="Y2" t="n">
-        <v>23.31328380098466</v>
+      <c r="AA2" t="n">
+        <v>23.31328394075086</v>
       </c>
     </row>
     <row r="3">
@@ -697,28 +713,34 @@
         <v>0.1065167260919373</v>
       </c>
       <c r="R3" t="n">
+        <v>0.06664459174752829</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.3263690029582119</v>
+      </c>
+      <c r="T3" t="n">
         <v>23.07142857142841</v>
       </c>
-      <c r="S3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" t="n">
-        <v>26.81456003824498</v>
-      </c>
       <c r="U3" t="n">
-        <v>1.851713165069686</v>
+        <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>0.006079853433416887</v>
+        <v>26.81456869324099</v>
       </c>
       <c r="W3" t="n">
-        <v>0.1278640288312575</v>
+        <v>1.851713413179842</v>
       </c>
       <c r="X3" t="n">
+        <v>0.006093564436306846</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0.1282317294427486</v>
+      </c>
+      <c r="Z3" t="n">
         <v>0.002428333333333334</v>
       </c>
-      <c r="Y3" t="n">
-        <v>26.65401311124306</v>
+      <c r="AA3" t="n">
+        <v>26.65401336848298</v>
       </c>
     </row>
     <row r="4">
@@ -780,28 +802,34 @@
         <v>0.08474551698518029</v>
       </c>
       <c r="R4" t="n">
+        <v>0.0585577437900562</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.2911108328200452</v>
+      </c>
+      <c r="T4" t="n">
         <v>23.9821428571428</v>
       </c>
-      <c r="S4" t="n">
+      <c r="U4" t="n">
         <v>0.1310102834270957</v>
       </c>
-      <c r="T4" t="n">
-        <v>27.04656525594052</v>
-      </c>
-      <c r="U4" t="n">
-        <v>1.856115873403019</v>
-      </c>
       <c r="V4" t="n">
-        <v>0.006462808694442893</v>
+        <v>27.04657382863489</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1368620630507388</v>
+        <v>1.856116121454714</v>
       </c>
       <c r="X4" t="n">
+        <v>0.006462750056087044</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0.1368605255335975</v>
+      </c>
+      <c r="Z4" t="n">
         <v>0.002603333333333333</v>
       </c>
-      <c r="Y4" t="n">
-        <v>26.81456003824498</v>
+      <c r="AA4" t="n">
+        <v>26.81456869324099</v>
       </c>
     </row>
     <row r="5">
@@ -863,28 +891,34 @@
         <v>0.06448817748780201</v>
       </c>
       <c r="R5" t="n">
+        <v>0.05054056312736721</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0.2539452253691769</v>
+      </c>
+      <c r="T5" t="n">
         <v>24.71428571428569</v>
       </c>
-      <c r="S5" t="n">
+      <c r="U5" t="n">
         <v>0.3150449672599142</v>
       </c>
-      <c r="T5" t="n">
-        <v>27.34710021604569</v>
-      </c>
-      <c r="U5" t="n">
-        <v>1.861850276180797</v>
-      </c>
       <c r="V5" t="n">
-        <v>0.006889873878741359</v>
+        <v>27.34710868323887</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1470709834936617</v>
+        <v>1.861850524232492</v>
       </c>
       <c r="X5" t="n">
+        <v>0.006890040482292315</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.1470755906637241</v>
+      </c>
+      <c r="Z5" t="n">
         <v>0.002815</v>
       </c>
-      <c r="Y5" t="n">
-        <v>27.04656525594052</v>
+      <c r="AA5" t="n">
+        <v>27.04657382863489</v>
       </c>
     </row>
     <row r="6">
@@ -946,28 +980,34 @@
         <v>0.112121445976553</v>
       </c>
       <c r="R6" t="n">
+        <v>0.06466559242177924</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.3348454060854844</v>
+      </c>
+      <c r="T6" t="n">
         <v>25.24642857142839</v>
       </c>
-      <c r="S6" t="n">
+      <c r="U6" t="n">
         <v>0.462353720667521</v>
       </c>
-      <c r="T6" t="n">
-        <v>27.65075345661634</v>
-      </c>
-      <c r="U6" t="n">
-        <v>1.867680276180797</v>
-      </c>
       <c r="V6" t="n">
-        <v>0.007276059687110452</v>
+        <v>27.65076181827065</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1565518660143671</v>
+        <v>1.867680524232492</v>
       </c>
       <c r="X6" t="n">
+        <v>0.007275870207412934</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0.1565466800263603</v>
+      </c>
+      <c r="Z6" t="n">
         <v>0.003015</v>
       </c>
-      <c r="Y6" t="n">
-        <v>27.34710021604569</v>
+      <c r="AA6" t="n">
+        <v>27.34710868323887</v>
       </c>
     </row>
     <row r="7">
@@ -1029,28 +1069,34 @@
         <v>0.2218548813486614</v>
       </c>
       <c r="R7" t="n">
+        <v>0.0901238156173267</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0.4710147358084048</v>
+      </c>
+      <c r="T7" t="n">
         <v>26.8128</v>
       </c>
-      <c r="S7" t="n">
+      <c r="U7" t="n">
         <v>0.6209461221159972</v>
       </c>
-      <c r="T7" t="n">
-        <v>27.96486690381572</v>
-      </c>
-      <c r="U7" t="n">
-        <v>1.873749651180797</v>
-      </c>
       <c r="V7" t="n">
-        <v>0.007634494500556047</v>
+        <v>27.96487515706328</v>
       </c>
       <c r="W7" t="n">
-        <v>0.1655898230009548</v>
+        <v>1.873749899232492</v>
       </c>
       <c r="X7" t="n">
+        <v>0.007634523293687587</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>0.1655906834098245</v>
+      </c>
+      <c r="Z7" t="n">
         <v>0.003210000000000001</v>
       </c>
-      <c r="Y7" t="n">
-        <v>27.65075345661634</v>
+      <c r="AA7" t="n">
+        <v>27.65076181827065</v>
       </c>
     </row>
     <row r="8">
@@ -1112,28 +1158,34 @@
         <v>0.3242312467603854</v>
       </c>
       <c r="R8" t="n">
+        <v>0.1082808906095662</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0.5694130721720264</v>
+      </c>
+      <c r="T8" t="n">
         <v>27.31428571428567</v>
       </c>
-      <c r="S8" t="n">
+      <c r="U8" t="n">
         <v>0.9523209449429346</v>
       </c>
-      <c r="T8" t="n">
-        <v>28.14125939280519</v>
-      </c>
-      <c r="U8" t="n">
-        <v>1.877175276180797</v>
-      </c>
       <c r="V8" t="n">
-        <v>0.007820573031697493</v>
+        <v>28.14126758547796</v>
       </c>
       <c r="W8" t="n">
-        <v>0.1703846824654642</v>
+        <v>1.877175524232492</v>
       </c>
       <c r="X8" t="n">
+        <v>0.007820569623933762</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>0.1703846427370974</v>
+      </c>
+      <c r="Z8" t="n">
         <v>0.003315</v>
       </c>
-      <c r="Y8" t="n">
-        <v>27.96486690381572</v>
+      <c r="AA8" t="n">
+        <v>27.96487515706328</v>
       </c>
     </row>
     <row r="9">
@@ -1195,28 +1247,34 @@
         <v>0.4847102107155994</v>
       </c>
       <c r="R9" t="n">
+        <v>0.1314793690318168</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0.6962113261902592</v>
+      </c>
+      <c r="T9" t="n">
         <v>27.65357142857139</v>
       </c>
-      <c r="S9" t="n">
+      <c r="U9" t="n">
         <v>1.25504016023201</v>
       </c>
-      <c r="T9" t="n">
-        <v>28.31682006754251</v>
-      </c>
-      <c r="U9" t="n">
-        <v>1.880597206736353</v>
-      </c>
       <c r="V9" t="n">
-        <v>0.007995870233119741</v>
+        <v>28.31682820030403</v>
       </c>
       <c r="W9" t="n">
-        <v>0.1749716551880656</v>
+        <v>1.880597454788048</v>
       </c>
       <c r="X9" t="n">
+        <v>0.007995866882157202</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>0.1749716173380987</v>
+      </c>
+      <c r="Z9" t="n">
         <v>0.003416666666666667</v>
       </c>
-      <c r="Y9" t="n">
-        <v>28.14125939280519</v>
+      <c r="AA9" t="n">
+        <v>28.14126758547796</v>
       </c>
     </row>
     <row r="10">
@@ -1278,28 +1336,34 @@
         <v>0.6709707039456413</v>
       </c>
       <c r="R10" t="n">
+        <v>0.153658332461822</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0.8191280143821486</v>
+      </c>
+      <c r="T10" t="n">
         <v>28.03928571428575</v>
       </c>
-      <c r="S10" t="n">
+      <c r="U10" t="n">
         <v>1.69587337268752</v>
       </c>
-      <c r="T10" t="n">
-        <v>28.48804706694351</v>
-      </c>
-      <c r="U10" t="n">
-        <v>1.883946706736353</v>
-      </c>
       <c r="V10" t="n">
-        <v>0.008158145764426144</v>
+        <v>28.48805514192954</v>
       </c>
       <c r="W10" t="n">
-        <v>0.1792828694645364</v>
+        <v>1.883946954788048</v>
       </c>
       <c r="X10" t="n">
+        <v>0.008158142377838717</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>0.1792828308002749</v>
+      </c>
+      <c r="Z10" t="n">
         <v>0.003513333333333334</v>
       </c>
-      <c r="Y10" t="n">
-        <v>28.31682006754251</v>
+      <c r="AA10" t="n">
+        <v>28.31682820030403</v>
       </c>
     </row>
     <row r="11">
@@ -1361,28 +1425,34 @@
         <v>0.1619956336149481</v>
       </c>
       <c r="R11" t="n">
+        <v>0.07756128526809224</v>
+      </c>
+      <c r="S11" t="n">
+        <v>0.4024868117279722</v>
+      </c>
+      <c r="T11" t="n">
         <v>26.35714285714281</v>
       </c>
-      <c r="S11" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" t="n">
-        <v>27.23145296079409</v>
-      </c>
       <c r="U11" t="n">
-        <v>1.90800233686873</v>
+        <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>0.01870831010401795</v>
+        <v>27.23145296063369</v>
       </c>
       <c r="W11" t="n">
-        <v>0.3981310530798082</v>
+        <v>1.908002336883929</v>
       </c>
       <c r="X11" t="n">
+        <v>0.01870851914241778</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>0.3981367454977016</v>
+      </c>
+      <c r="Z11" t="n">
         <v>0.007799999999999998</v>
       </c>
-      <c r="Y11" t="n">
-        <v>26.32781437148795</v>
+      <c r="AA11" t="n">
+        <v>26.32781445538231</v>
       </c>
     </row>
     <row r="12">
@@ -1444,28 +1514,34 @@
         <v>0.0921971490896749</v>
       </c>
       <c r="R12" t="n">
+        <v>0.06022672929531771</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0.3036398344909226</v>
+      </c>
+      <c r="T12" t="n">
         <v>26.92857142857148</v>
       </c>
-      <c r="S12" t="n">
+      <c r="U12" t="n">
         <v>0.1961577414134905</v>
       </c>
-      <c r="T12" t="n">
-        <v>27.96947227861317</v>
-      </c>
-      <c r="U12" t="n">
-        <v>1.92257108686873</v>
-      </c>
       <c r="V12" t="n">
-        <v>0.02051071490900611</v>
+        <v>27.9694722689493</v>
       </c>
       <c r="W12" t="n">
-        <v>0.4449244950655394</v>
+        <v>1.922571086883929</v>
       </c>
       <c r="X12" t="n">
+        <v>0.02051073157175735</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>0.4449249609611882</v>
+      </c>
+      <c r="Z12" t="n">
         <v>0.008849999999999998</v>
       </c>
-      <c r="Y12" t="n">
-        <v>27.23145296079409</v>
+      <c r="AA12" t="n">
+        <v>27.23145296063369</v>
       </c>
     </row>
     <row r="13">
@@ -1521,34 +1597,40 @@
         <v>0.006274829559544594</v>
       </c>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q13" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R13" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S13" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T13" t="n">
         <v>25.41785714285721</v>
       </c>
-      <c r="S13" t="n">
+      <c r="U13" t="n">
         <v>0.4648676866334254</v>
       </c>
-      <c r="T13" t="n">
-        <v>28.96836793855088</v>
-      </c>
-      <c r="U13" t="n">
-        <v>1.942647670202063</v>
-      </c>
       <c r="V13" t="n">
-        <v>0.02241121869123013</v>
+        <v>28.96836727463392</v>
       </c>
       <c r="W13" t="n">
-        <v>0.498309042119181</v>
+        <v>1.942647670217263</v>
       </c>
       <c r="X13" t="n">
+        <v>0.02241123524433885</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>0.4983095102163055</v>
+      </c>
+      <c r="Z13" t="n">
         <v>0.01012</v>
       </c>
-      <c r="Y13" t="n">
-        <v>27.96947227861317</v>
+      <c r="AA13" t="n">
+        <v>27.9694722689493</v>
       </c>
     </row>
     <row r="14">
@@ -1610,28 +1692,34 @@
         <v>0.166038915540943</v>
       </c>
       <c r="R14" t="n">
+        <v>0.07737225717069976</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0.4074787301699844</v>
+      </c>
+      <c r="T14" t="n">
         <v>27.31785714285721</v>
       </c>
-      <c r="S14" t="n">
+      <c r="U14" t="n">
         <v>0.5273275582417261</v>
       </c>
-      <c r="T14" t="n">
-        <v>30.012551032435</v>
-      </c>
-      <c r="U14" t="n">
-        <v>1.964087670202063</v>
-      </c>
       <c r="V14" t="n">
-        <v>0.02393237134192201</v>
+        <v>30.01254965667641</v>
       </c>
       <c r="W14" t="n">
-        <v>0.5452944730724245</v>
+        <v>1.964087670217262</v>
       </c>
       <c r="X14" t="n">
+        <v>0.02393238700794108</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>0.5452949182549442</v>
+      </c>
+      <c r="Z14" t="n">
         <v>0.01132</v>
       </c>
-      <c r="Y14" t="n">
-        <v>28.96836793855088</v>
+      <c r="AA14" t="n">
+        <v>28.96836727463392</v>
       </c>
     </row>
     <row r="15">
@@ -1693,28 +1781,34 @@
         <v>0.6940734053890505</v>
       </c>
       <c r="R15" t="n">
+        <v>0.1504129176969866</v>
+      </c>
+      <c r="S15" t="n">
+        <v>0.8331106801554344</v>
+      </c>
+      <c r="T15" t="n">
         <v>27.73571428571431</v>
       </c>
-      <c r="S15" t="n">
+      <c r="U15" t="n">
         <v>0.5669120469218694</v>
       </c>
-      <c r="T15" t="n">
-        <v>31.10797224513737</v>
-      </c>
-      <c r="U15" t="n">
-        <v>1.98709433686873</v>
-      </c>
       <c r="V15" t="n">
-        <v>0.02516111466725047</v>
+        <v>31.10797015051896</v>
       </c>
       <c r="W15" t="n">
-        <v>0.5873367913989104</v>
+        <v>1.987094336883929</v>
       </c>
       <c r="X15" t="n">
+        <v>0.02516114519472265</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>0.5873377015004719</v>
+      </c>
+      <c r="Z15" t="n">
         <v>0.01248</v>
       </c>
-      <c r="Y15" t="n">
-        <v>30.012551032435</v>
+      <c r="AA15" t="n">
+        <v>30.01254965667641</v>
       </c>
     </row>
     <row r="16">
@@ -1776,28 +1870,34 @@
         <v>1.033509465599738</v>
       </c>
       <c r="R16" t="n">
+        <v>0.1835437763974597</v>
+      </c>
+      <c r="S16" t="n">
+        <v>1.016616675841852</v>
+      </c>
+      <c r="T16" t="n">
         <v>30.67857142857135</v>
       </c>
-      <c r="S16" t="n">
+      <c r="U16" t="n">
         <v>1.314363106233276</v>
       </c>
-      <c r="T16" t="n">
-        <v>31.7461397651932</v>
-      </c>
-      <c r="U16" t="n">
-        <v>2.000747670202063</v>
-      </c>
       <c r="V16" t="n">
-        <v>0.02574269341415964</v>
+        <v>31.74613730418875</v>
       </c>
       <c r="W16" t="n">
-        <v>0.6090542900136535</v>
+        <v>2.000747670217262</v>
       </c>
       <c r="X16" t="n">
+        <v>0.02574269542905198</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>0.6090543067655569</v>
+      </c>
+      <c r="Z16" t="n">
         <v>0.01312</v>
       </c>
-      <c r="Y16" t="n">
-        <v>31.10797224513737</v>
+      <c r="AA16" t="n">
+        <v>31.10797015051896</v>
       </c>
     </row>
     <row r="17">
@@ -1859,28 +1959,34 @@
         <v>0.0816312894067058</v>
       </c>
       <c r="R17" t="n">
+        <v>0.05155349562266365</v>
+      </c>
+      <c r="S17" t="n">
+        <v>0.2857118993089119</v>
+      </c>
+      <c r="T17" t="n">
         <v>29.52857142857138</v>
       </c>
-      <c r="S17" t="n">
-        <v>0</v>
-      </c>
-      <c r="T17" t="n">
-        <v>19.99434722561607</v>
-      </c>
       <c r="U17" t="n">
-        <v>1.878764027797204</v>
+        <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>0.006624136125296541</v>
+        <v>19.9943493428161</v>
       </c>
       <c r="W17" t="n">
-        <v>0.1111961767348054</v>
+        <v>1.878764110411336</v>
       </c>
       <c r="X17" t="n">
+        <v>0.006624133662702124</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>0.1111961402057659</v>
+      </c>
+      <c r="Z17" t="n">
         <v>0.001996666666666667</v>
       </c>
-      <c r="Y17" t="n">
-        <v>16.88071097278224</v>
+      <c r="AA17" t="n">
+        <v>16.88071214887976</v>
       </c>
     </row>
     <row r="18">
@@ -1942,28 +2048,34 @@
         <v>0.04078878183453907</v>
       </c>
       <c r="R18" t="n">
+        <v>0.0359356095867547</v>
+      </c>
+      <c r="S18" t="n">
+        <v>0.2019623277607462</v>
+      </c>
+      <c r="T18" t="n">
         <v>30.71428571428574</v>
       </c>
-      <c r="S18" t="n">
+      <c r="U18" t="n">
         <v>0.09290978010103844</v>
       </c>
-      <c r="T18" t="n">
-        <v>20.11820097131467</v>
-      </c>
-      <c r="U18" t="n">
-        <v>1.880990611130537</v>
-      </c>
       <c r="V18" t="n">
-        <v>0.006756799854998181</v>
+        <v>20.1182030731978</v>
       </c>
       <c r="W18" t="n">
-        <v>0.1139909847038225</v>
+        <v>1.88099069374467</v>
       </c>
       <c r="X18" t="n">
+        <v>0.006756696680435864</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>0.1139889218902052</v>
+      </c>
+      <c r="Z18" t="n">
         <v>0.002051666666666667</v>
       </c>
-      <c r="Y18" t="n">
-        <v>19.99434722561607</v>
+      <c r="AA18" t="n">
+        <v>19.9943493428161</v>
       </c>
     </row>
     <row r="19">
@@ -2025,28 +2137,34 @@
         <v>0.02413582546819065</v>
       </c>
       <c r="R19" t="n">
+        <v>0.02706031021828268</v>
+      </c>
+      <c r="S19" t="n">
+        <v>0.1553570901767623</v>
+      </c>
+      <c r="T19" t="n">
         <v>31.58571428571431</v>
       </c>
-      <c r="S19" t="n">
+      <c r="U19" t="n">
         <v>0.1714635834683609</v>
       </c>
-      <c r="T19" t="n">
-        <v>20.22568990616278</v>
-      </c>
-      <c r="U19" t="n">
-        <v>1.882927277797204</v>
-      </c>
       <c r="V19" t="n">
-        <v>0.006866587876487551</v>
+        <v>20.22569199499107</v>
       </c>
       <c r="W19" t="n">
-        <v>0.1163419771341342</v>
+        <v>1.882927360411336</v>
       </c>
       <c r="X19" t="n">
+        <v>0.006866586904202878</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>0.1163419704732665</v>
+      </c>
+      <c r="Z19" t="n">
         <v>0.002098333333333333</v>
       </c>
-      <c r="Y19" t="n">
-        <v>20.11820097131467</v>
+      <c r="AA19" t="n">
+        <v>20.1182030731978</v>
       </c>
     </row>
     <row r="20">
@@ -2108,28 +2226,34 @@
         <v>0.03974752399441857</v>
       </c>
       <c r="R20" t="n">
+        <v>0.03441311909386455</v>
+      </c>
+      <c r="S20" t="n">
+        <v>0.199367810828174</v>
+      </c>
+      <c r="T20" t="n">
         <v>32.96071428571437</v>
       </c>
-      <c r="S20" t="n">
+      <c r="U20" t="n">
         <v>0.1940649581558863</v>
       </c>
-      <c r="T20" t="n">
-        <v>20.34328539823888</v>
-      </c>
-      <c r="U20" t="n">
-        <v>1.885050611130537</v>
-      </c>
       <c r="V20" t="n">
-        <v>0.006981703852210943</v>
+        <v>20.34328747236598</v>
       </c>
       <c r="W20" t="n">
-        <v>0.1188461867469677</v>
+        <v>1.88505069374467</v>
       </c>
       <c r="X20" t="n">
+        <v>0.006981715983853094</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>0.1188464466776623</v>
+      </c>
+      <c r="Z20" t="n">
         <v>0.002148333333333333</v>
       </c>
-      <c r="Y20" t="n">
-        <v>20.22568990616278</v>
+      <c r="AA20" t="n">
+        <v>20.22569199499107</v>
       </c>
     </row>
     <row r="21">
@@ -2191,28 +2315,34 @@
         <v>0.07526448485171559</v>
       </c>
       <c r="R21" t="n">
+        <v>0.04747282035761839</v>
+      </c>
+      <c r="S21" t="n">
+        <v>0.2743437348504894</v>
+      </c>
+      <c r="T21" t="n">
         <v>33.56309523809537</v>
       </c>
-      <c r="S21" t="n">
+      <c r="U21" t="n">
         <v>0.2229784488956445</v>
       </c>
-      <c r="T21" t="n">
-        <v>20.4734955867161</v>
-      </c>
-      <c r="U21" t="n">
-        <v>1.887407312519426</v>
-      </c>
       <c r="V21" t="n">
-        <v>0.007103353408241623</v>
+        <v>20.47349764508844</v>
       </c>
       <c r="W21" t="n">
-        <v>0.1215390370561618</v>
+        <v>1.887407395133558</v>
       </c>
       <c r="X21" t="n">
+        <v>0.007103342896403787</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>0.1215388351071716</v>
+      </c>
+      <c r="Z21" t="n">
         <v>0.0022025</v>
       </c>
-      <c r="Y21" t="n">
-        <v>20.34328539823888</v>
+      <c r="AA21" t="n">
+        <v>20.34328747236598</v>
       </c>
     </row>
     <row r="22">
@@ -2274,28 +2404,34 @@
         <v>0.102602067198723</v>
       </c>
       <c r="R22" t="n">
+        <v>0.05491924762933701</v>
+      </c>
+      <c r="S22" t="n">
+        <v>0.3203155743930086</v>
+      </c>
+      <c r="T22" t="n">
         <v>33.39642857142849</v>
       </c>
-      <c r="S22" t="n">
+      <c r="U22" t="n">
         <v>0.2989185664601128</v>
       </c>
-      <c r="T22" t="n">
-        <v>20.58181820907232</v>
-      </c>
-      <c r="U22" t="n">
-        <v>1.889372361130537</v>
-      </c>
       <c r="V22" t="n">
-        <v>0.007200136730610088</v>
+        <v>20.58182025443793</v>
       </c>
       <c r="W22" t="n">
-        <v>0.1237179128155578</v>
+        <v>1.889372443744669</v>
       </c>
       <c r="X22" t="n">
+        <v>0.007200135700517285</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>0.1237179049792681</v>
+      </c>
+      <c r="Z22" t="n">
         <v>0.002246666666666667</v>
       </c>
-      <c r="Y22" t="n">
-        <v>20.4734955867161</v>
+      <c r="AA22" t="n">
+        <v>20.47349764508844</v>
       </c>
     </row>
     <row r="23">
@@ -2357,28 +2493,34 @@
         <v>0.06320238611045444</v>
       </c>
       <c r="R23" t="n">
+        <v>0.0464330358326207</v>
+      </c>
+      <c r="S23" t="n">
+        <v>0.2514008474736202</v>
+      </c>
+      <c r="T23" t="n">
         <v>28.42857142857147</v>
       </c>
-      <c r="S23" t="n">
-        <v>0</v>
-      </c>
-      <c r="T23" t="n">
-        <v>15.01969250760888</v>
-      </c>
       <c r="U23" t="n">
-        <v>1.792146527764305</v>
+        <v>0</v>
       </c>
       <c r="V23" t="n">
-        <v>0.009244326228632355</v>
+        <v>15.01969296805368</v>
       </c>
       <c r="W23" t="n">
-        <v>0.1221131944166381</v>
+        <v>1.792146539303604</v>
       </c>
       <c r="X23" t="n">
+        <v>0.00924435718584087</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>0.1221136632356617</v>
+      </c>
+      <c r="Z23" t="n">
         <v>0.001996666666666667</v>
       </c>
-      <c r="Y23" t="n">
-        <v>14.80438644777559</v>
+      <c r="AA23" t="n">
+        <v>14.80438687360635</v>
       </c>
     </row>
     <row r="24">
@@ -2440,28 +2582,34 @@
         <v>0.05093049240086417</v>
       </c>
       <c r="R24" t="n">
+        <v>0.04115887469949947</v>
+      </c>
+      <c r="S24" t="n">
+        <v>0.2256778509310654</v>
+      </c>
+      <c r="T24" t="n">
         <v>29.31428571428569</v>
       </c>
-      <c r="S24" t="n">
+      <c r="U24" t="n">
         <v>0.05810793948216079</v>
       </c>
-      <c r="T24" t="n">
-        <v>15.15569778641188</v>
-      </c>
-      <c r="U24" t="n">
-        <v>1.794373111097638</v>
-      </c>
       <c r="V24" t="n">
-        <v>0.009401995746227973</v>
+        <v>15.15569823705797</v>
       </c>
       <c r="W24" t="n">
-        <v>0.1251649463817385</v>
+        <v>1.794373122636937</v>
       </c>
       <c r="X24" t="n">
+        <v>0.00940201309158991</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>0.1251652130959574</v>
+      </c>
+      <c r="Z24" t="n">
         <v>0.002051666666666667</v>
       </c>
-      <c r="Y24" t="n">
-        <v>15.01969250760888</v>
+      <c r="AA24" t="n">
+        <v>15.01969296805368</v>
       </c>
     </row>
     <row r="25">
@@ -2523,28 +2671,34 @@
         <v>0.03650228328522884</v>
       </c>
       <c r="R25" t="n">
+        <v>0.03434893131725996</v>
+      </c>
+      <c r="S25" t="n">
+        <v>0.1910557072825328</v>
+      </c>
+      <c r="T25" t="n">
         <v>30.06428571428577</v>
       </c>
-      <c r="S25" t="n">
+      <c r="U25" t="n">
         <v>0.1219400842896329</v>
       </c>
-      <c r="T25" t="n">
-        <v>15.27797946826978</v>
-      </c>
-      <c r="U25" t="n">
-        <v>1.796379749986527</v>
-      </c>
       <c r="V25" t="n">
-        <v>0.009535924639375432</v>
+        <v>15.27797991000348</v>
       </c>
       <c r="W25" t="n">
-        <v>0.12782943008243</v>
+        <v>1.796379761525826</v>
       </c>
       <c r="X25" t="n">
+        <v>0.009535909472786619</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>0.1278292021782632</v>
+      </c>
+      <c r="Z25" t="n">
         <v>0.0021</v>
       </c>
-      <c r="Y25" t="n">
-        <v>15.15569778641188</v>
+      <c r="AA25" t="n">
+        <v>15.15569823705797</v>
       </c>
     </row>
     <row r="26">
@@ -2606,28 +2760,34 @@
         <v>0.01662203559450923</v>
       </c>
       <c r="R26" t="n">
+        <v>0.02296789446903608</v>
+      </c>
+      <c r="S26" t="n">
+        <v>0.1289264735983624</v>
+      </c>
+      <c r="T26" t="n">
         <v>30.93809523809523</v>
       </c>
-      <c r="S26" t="n">
+      <c r="U26" t="n">
         <v>0.1703755277559266</v>
       </c>
-      <c r="T26" t="n">
-        <v>15.40717642178005</v>
-      </c>
-      <c r="U26" t="n">
-        <v>1.798504749986527</v>
-      </c>
       <c r="V26" t="n">
-        <v>0.009669490718981348</v>
+        <v>15.40717685453495</v>
       </c>
       <c r="W26" t="n">
-        <v>0.1305612331413965</v>
+        <v>1.798504761525826</v>
       </c>
       <c r="X26" t="n">
+        <v>0.009669568421304507</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>0.1305624341001924</v>
+      </c>
+      <c r="Z26" t="n">
         <v>0.00215</v>
       </c>
-      <c r="Y26" t="n">
-        <v>15.27797946826978</v>
+      <c r="AA26" t="n">
+        <v>15.27797991000348</v>
       </c>
     </row>
     <row r="27">
@@ -2683,34 +2843,40 @@
         <v>0</v>
       </c>
       <c r="P27" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q27" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R27" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S27" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T27" t="n">
         <v>31.5095238095239</v>
       </c>
-      <c r="S27" t="n">
+      <c r="U27" t="n">
         <v>0.2036432131066642</v>
       </c>
-      <c r="T27" t="n">
-        <v>15.54576471769251</v>
-      </c>
-      <c r="U27" t="n">
-        <v>1.800789812486527</v>
-      </c>
       <c r="V27" t="n">
-        <v>0.009804969956134207</v>
+        <v>15.54576514061194</v>
       </c>
       <c r="W27" t="n">
-        <v>0.1334121284519593</v>
+        <v>1.800789824025826</v>
       </c>
       <c r="X27" t="n">
+        <v>0.009804949344494194</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>0.1334118117795324</v>
+      </c>
+      <c r="Z27" t="n">
         <v>0.0022025</v>
       </c>
-      <c r="Y27" t="n">
-        <v>15.40717642178005</v>
+      <c r="AA27" t="n">
+        <v>15.40717685453495</v>
       </c>
     </row>
     <row r="28">
@@ -2766,34 +2932,40 @@
         <v>0.07036365759109456</v>
       </c>
       <c r="P28" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q28" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R28" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S28" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T28" t="n">
         <v>31.73214285714281</v>
       </c>
-      <c r="S28" t="n">
+      <c r="U28" t="n">
         <v>0.2220723133576301</v>
       </c>
-      <c r="T28" t="n">
-        <v>15.66240050531441</v>
-      </c>
-      <c r="U28" t="n">
-        <v>1.802717423597638</v>
-      </c>
       <c r="V28" t="n">
-        <v>0.009912768036938789</v>
+        <v>15.66240091965512</v>
       </c>
       <c r="W28" t="n">
-        <v>0.1357454553421338</v>
+        <v>1.802717435136937</v>
       </c>
       <c r="X28" t="n">
+        <v>0.009912767707050024</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>0.1357454538912589</v>
+      </c>
+      <c r="Z28" t="n">
         <v>0.002245833333333333</v>
       </c>
-      <c r="Y28" t="n">
-        <v>15.54576471769251</v>
+      <c r="AA28" t="n">
+        <v>15.54576514061194</v>
       </c>
     </row>
     <row r="29">
@@ -2855,28 +3027,34 @@
         <v>0.07399229663180125</v>
       </c>
       <c r="R29" t="n">
+        <v>0.05414454690340646</v>
+      </c>
+      <c r="S29" t="n">
+        <v>0.2720152507338536</v>
+      </c>
+      <c r="T29" t="n">
         <v>24.49345238095237</v>
       </c>
-      <c r="S29" t="n">
-        <v>0</v>
-      </c>
-      <c r="T29" t="n">
-        <v>23.93967898585161</v>
-      </c>
       <c r="U29" t="n">
-        <v>2.098491694450313</v>
+        <v>0</v>
       </c>
       <c r="V29" t="n">
-        <v>0.01007971427442612</v>
+        <v>23.93968006453909</v>
       </c>
       <c r="W29" t="n">
-        <v>0.1949504513214563</v>
+        <v>2.098491720806879</v>
       </c>
       <c r="X29" t="n">
+        <v>0.01007997637280434</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>0.194956735239167</v>
+      </c>
+      <c r="Z29" t="n">
         <v>0.004063333333333333</v>
       </c>
-      <c r="Y29" t="n">
-        <v>23.76781114604884</v>
+      <c r="AA29" t="n">
+        <v>23.76781203213405</v>
       </c>
     </row>
     <row r="30">
@@ -2938,28 +3116,34 @@
         <v>0.06485638924285067</v>
       </c>
       <c r="R30" t="n">
+        <v>0.05116644028606399</v>
+      </c>
+      <c r="S30" t="n">
+        <v>0.2546691760752578</v>
+      </c>
+      <c r="T30" t="n">
         <v>25.23928571428564</v>
       </c>
-      <c r="S30" t="n">
+      <c r="U30" t="n">
         <v>0.06375494686076261</v>
       </c>
-      <c r="T30" t="n">
-        <v>24.22814583641843</v>
-      </c>
-      <c r="U30" t="n">
-        <v>2.104521250005869</v>
-      </c>
       <c r="V30" t="n">
-        <v>0.01063211796426457</v>
+        <v>24.22814684652792</v>
       </c>
       <c r="W30" t="n">
-        <v>0.2075174500820442</v>
+        <v>2.104521276362434</v>
       </c>
       <c r="X30" t="n">
+        <v>0.01063212456913026</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>0.207517619384608</v>
+      </c>
+      <c r="Z30" t="n">
         <v>0.00435</v>
       </c>
-      <c r="Y30" t="n">
-        <v>23.93967898585161</v>
+      <c r="AA30" t="n">
+        <v>23.93968006453909</v>
       </c>
     </row>
     <row r="31">
@@ -3021,28 +3205,34 @@
         <v>0.04872158819598323</v>
       </c>
       <c r="R31" t="n">
+        <v>0.0441207297966015</v>
+      </c>
+      <c r="S31" t="n">
+        <v>0.2207296722146418</v>
+      </c>
+      <c r="T31" t="n">
         <v>24.77321428571426</v>
       </c>
-      <c r="S31" t="n">
+      <c r="U31" t="n">
         <v>0.1716212668026328</v>
       </c>
-      <c r="T31" t="n">
-        <v>24.54912557034737</v>
-      </c>
-      <c r="U31" t="n">
-        <v>2.111271250005868</v>
-      </c>
       <c r="V31" t="n">
-        <v>0.01118089966425217</v>
+        <v>24.54912650345894</v>
       </c>
       <c r="W31" t="n">
-        <v>0.22041273201674</v>
+        <v>2.111271276362434</v>
       </c>
       <c r="X31" t="n">
+        <v>0.01118092410442565</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>0.2204133410545105</v>
+      </c>
+      <c r="Z31" t="n">
         <v>0.00465</v>
       </c>
-      <c r="Y31" t="n">
-        <v>24.22814583641843</v>
+      <c r="AA31" t="n">
+        <v>24.22814684652792</v>
       </c>
     </row>
     <row r="32">
@@ -3104,28 +3294,34 @@
         <v>0.03284030984725474</v>
       </c>
       <c r="R32" t="n">
+        <v>0.03536550708002241</v>
+      </c>
+      <c r="S32" t="n">
+        <v>0.1812189555406794</v>
+      </c>
+      <c r="T32" t="n">
         <v>25.0285714285714</v>
       </c>
-      <c r="S32" t="n">
+      <c r="U32" t="n">
         <v>0.2547670720457892</v>
       </c>
-      <c r="T32" t="n">
-        <v>25.00680786787553</v>
-      </c>
-      <c r="U32" t="n">
-        <v>2.120971250005868</v>
-      </c>
       <c r="V32" t="n">
-        <v>0.0118658838353382</v>
+        <v>25.00680869176568</v>
       </c>
       <c r="W32" t="n">
-        <v>0.2371870514484175</v>
+        <v>2.120971276362434</v>
       </c>
       <c r="X32" t="n">
+        <v>0.01186587573608902</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>0.2371868574664508</v>
+      </c>
+      <c r="Z32" t="n">
         <v>0.005050000000000001</v>
       </c>
-      <c r="Y32" t="n">
-        <v>24.54912557034737</v>
+      <c r="AA32" t="n">
+        <v>24.54912650345894</v>
       </c>
     </row>
     <row r="33">
@@ -3187,28 +3383,34 @@
         <v>0.002777158124534164</v>
       </c>
       <c r="R33" t="n">
+        <v>0.01006757845422143</v>
+      </c>
+      <c r="S33" t="n">
+        <v>0.05269874879476897</v>
+      </c>
+      <c r="T33" t="n">
         <v>26.25714285714279</v>
       </c>
-      <c r="S33" t="n">
+      <c r="U33" t="n">
         <v>0.3345630000595383</v>
       </c>
-      <c r="T33" t="n">
-        <v>26.11045456428113</v>
-      </c>
-      <c r="U33" t="n">
-        <v>2.14473236111698</v>
-      </c>
       <c r="V33" t="n">
-        <v>0.01316721393135566</v>
+        <v>26.11045512932166</v>
       </c>
       <c r="W33" t="n">
-        <v>0.2717711091938156</v>
+        <v>2.144732387473546</v>
       </c>
       <c r="X33" t="n">
+        <v>0.01316721250280378</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>0.271771078660095</v>
+      </c>
+      <c r="Z33" t="n">
         <v>0.005916666666666667</v>
       </c>
-      <c r="Y33" t="n">
-        <v>25.00680786787553</v>
+      <c r="AA33" t="n">
+        <v>25.00680869176568</v>
       </c>
     </row>
     <row r="34">
@@ -3264,34 +3466,40 @@
         <v>0.01145255846603085</v>
       </c>
       <c r="P34" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q34" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R34" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S34" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T34" t="n">
         <v>27.40000000000004</v>
       </c>
-      <c r="S34" t="n">
+      <c r="U34" t="n">
         <v>0.4114676331552647</v>
       </c>
-      <c r="T34" t="n">
-        <v>26.57397314631664</v>
-      </c>
-      <c r="U34" t="n">
-        <v>2.154871250005869</v>
-      </c>
       <c r="V34" t="n">
-        <v>0.01360205894586814</v>
+        <v>26.57397360426178</v>
       </c>
       <c r="W34" t="n">
-        <v>0.2843854565366162</v>
+        <v>2.154871276362434</v>
       </c>
       <c r="X34" t="n">
+        <v>0.01360205481603644</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>0.2843853526340677</v>
+      </c>
+      <c r="Z34" t="n">
         <v>0.00625</v>
       </c>
-      <c r="Y34" t="n">
-        <v>26.11045456428113</v>
+      <c r="AA34" t="n">
+        <v>26.11045512932166</v>
       </c>
     </row>
     <row r="35">
@@ -3353,28 +3561,34 @@
         <v>0.001762949417501451</v>
       </c>
       <c r="R35" t="n">
+        <v>0.007839965084997607</v>
+      </c>
+      <c r="S35" t="n">
+        <v>0.04198749120275527</v>
+      </c>
+      <c r="T35" t="n">
         <v>28.4607142857143</v>
       </c>
-      <c r="S35" t="n">
+      <c r="U35" t="n">
         <v>0.4067877264015557</v>
       </c>
-      <c r="T35" t="n">
-        <v>27.30784322886136</v>
-      </c>
-      <c r="U35" t="n">
-        <v>2.171121250005869</v>
-      </c>
       <c r="V35" t="n">
-        <v>0.01418844280408847</v>
+        <v>27.30784352193885</v>
       </c>
       <c r="W35" t="n">
-        <v>0.302555887977083</v>
+        <v>2.171121276362435</v>
       </c>
       <c r="X35" t="n">
+        <v>0.01418840491525607</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>0.3025548575925655</v>
+      </c>
+      <c r="Z35" t="n">
         <v>0.006750000000000001</v>
       </c>
-      <c r="Y35" t="n">
-        <v>26.57397314631664</v>
+      <c r="AA35" t="n">
+        <v>26.57397360426178</v>
       </c>
     </row>
     <row r="36">
@@ -3436,28 +3650,34 @@
         <v>0.001647154283060745</v>
       </c>
       <c r="R36" t="n">
+        <v>0.007564472262002585</v>
+      </c>
+      <c r="S36" t="n">
+        <v>0.04058514855289733</v>
+      </c>
+      <c r="T36" t="n">
         <v>28.6821428571429</v>
       </c>
-      <c r="S36" t="n">
+      <c r="U36" t="n">
         <v>0.4021708299263646</v>
       </c>
-      <c r="T36" t="n">
-        <v>27.82182632953165</v>
-      </c>
-      <c r="U36" t="n">
-        <v>2.182649027783647</v>
-      </c>
       <c r="V36" t="n">
-        <v>0.01453702929851717</v>
+        <v>27.82182651078572</v>
       </c>
       <c r="W36" t="n">
-        <v>0.31415675529333</v>
+        <v>2.182649054140212</v>
       </c>
       <c r="X36" t="n">
+        <v>0.01453692586273916</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>0.3141538806580285</v>
+      </c>
+      <c r="Z36" t="n">
         <v>0.007083333333333334</v>
       </c>
-      <c r="Y36" t="n">
-        <v>27.30784322886136</v>
+      <c r="AA36" t="n">
+        <v>27.30784352193885</v>
       </c>
     </row>
     <row r="37">
@@ -3519,28 +3739,34 @@
         <v>0.0005503013934911842</v>
       </c>
       <c r="R37" t="n">
+        <v>0.004370963058975695</v>
+      </c>
+      <c r="S37" t="n">
+        <v>0.02345850364987469</v>
+      </c>
+      <c r="T37" t="n">
         <v>28.78571428571429</v>
       </c>
-      <c r="S37" t="n">
+      <c r="U37" t="n">
         <v>0.3873938421634567</v>
       </c>
-      <c r="T37" t="n">
-        <v>28.72212538886001</v>
-      </c>
-      <c r="U37" t="n">
-        <v>2.203139000005869</v>
-      </c>
       <c r="V37" t="n">
-        <v>0.01504659646470858</v>
+        <v>28.72212537780479</v>
       </c>
       <c r="W37" t="n">
-        <v>0.3325682361029325</v>
+        <v>2.203139026362434</v>
       </c>
       <c r="X37" t="n">
+        <v>0.01504659517082482</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>0.3325682000033916</v>
+      </c>
+      <c r="Z37" t="n">
         <v>0.007640000000000001</v>
       </c>
-      <c r="Y37" t="n">
-        <v>27.82182632953165</v>
+      <c r="AA37" t="n">
+        <v>27.82182651078572</v>
       </c>
     </row>
     <row r="38">
@@ -3602,28 +3828,34 @@
         <v>0.0004247662125730495</v>
       </c>
       <c r="R38" t="n">
+        <v>0.003775433716909023</v>
+      </c>
+      <c r="S38" t="n">
+        <v>0.02060985717012735</v>
+      </c>
+      <c r="T38" t="n">
         <v>28.80357142857139</v>
       </c>
-      <c r="S38" t="n">
+      <c r="U38" t="n">
         <v>0.3689307159607038</v>
       </c>
-      <c r="T38" t="n">
-        <v>29.76547646662382</v>
-      </c>
-      <c r="U38" t="n">
-        <v>2.227371250005869</v>
-      </c>
       <c r="V38" t="n">
-        <v>0.01550780134710743</v>
+        <v>29.76547634687633</v>
       </c>
       <c r="W38" t="n">
-        <v>0.3513482182048674</v>
+        <v>2.227371276362434</v>
       </c>
       <c r="X38" t="n">
+        <v>0.01550781476267443</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>0.3513486174167029</v>
+      </c>
+      <c r="Z38" t="n">
         <v>0.00825</v>
       </c>
-      <c r="Y38" t="n">
-        <v>28.72212538886001</v>
+      <c r="AA38" t="n">
+        <v>28.72212537780479</v>
       </c>
     </row>
     <row r="39">
@@ -3685,28 +3917,34 @@
         <v>0.008954679612111731</v>
       </c>
       <c r="R39" t="n">
+        <v>0.01696173781741488</v>
+      </c>
+      <c r="S39" t="n">
+        <v>0.09462916892856943</v>
+      </c>
+      <c r="T39" t="n">
         <v>29.79999999999999</v>
       </c>
-      <c r="S39" t="n">
+      <c r="U39" t="n">
         <v>0.3542503465167628</v>
       </c>
-      <c r="T39" t="n">
-        <v>30.84541916586719</v>
-      </c>
-      <c r="U39" t="n">
-        <v>2.253021250005869</v>
-      </c>
       <c r="V39" t="n">
-        <v>0.01587052728317392</v>
+        <v>30.84541902494425</v>
       </c>
       <c r="W39" t="n">
-        <v>0.3683704455222586</v>
+        <v>2.253021276362434</v>
       </c>
       <c r="X39" t="n">
+        <v>0.01587053886464064</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>0.3683708024918843</v>
+      </c>
+      <c r="Z39" t="n">
         <v>0.00885</v>
       </c>
-      <c r="Y39" t="n">
-        <v>29.76547646662382</v>
+      <c r="AA39" t="n">
+        <v>29.76547634687633</v>
       </c>
     </row>
     <row r="40">
@@ -3768,28 +4006,34 @@
         <v>0.02192219084074996</v>
       </c>
       <c r="R40" t="n">
+        <v>0.02664331523520602</v>
+      </c>
+      <c r="S40" t="n">
+        <v>0.148061442788965</v>
+      </c>
+      <c r="T40" t="n">
         <v>31.12500000000002</v>
       </c>
-      <c r="S40" t="n">
+      <c r="U40" t="n">
         <v>0.363160750555521</v>
       </c>
-      <c r="T40" t="n">
-        <v>31.81469618095175</v>
-      </c>
-      <c r="U40" t="n">
-        <v>2.27655111111698</v>
-      </c>
       <c r="V40" t="n">
-        <v>0.01611696629351479</v>
+        <v>31.8146960202547</v>
       </c>
       <c r="W40" t="n">
-        <v>0.3818576537892139</v>
+        <v>2.276551137473545</v>
       </c>
       <c r="X40" t="n">
+        <v>0.01611696618632926</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>0.3818576499658321</v>
+      </c>
+      <c r="Z40" t="n">
         <v>0.009366666666666667</v>
       </c>
-      <c r="Y40" t="n">
-        <v>30.84541916586719</v>
+      <c r="AA40" t="n">
+        <v>30.84541902494425</v>
       </c>
     </row>
     <row r="41">
@@ -3851,28 +4095,34 @@
         <v>0.04292053230848831</v>
       </c>
       <c r="R41" t="n">
+        <v>0.03929002064237096</v>
+      </c>
+      <c r="S41" t="n">
+        <v>0.2071727113026431</v>
+      </c>
+      <c r="T41" t="n">
         <v>25.66428571428573</v>
       </c>
-      <c r="S41" t="n">
-        <v>0</v>
-      </c>
-      <c r="T41" t="n">
-        <v>28.24180486772746</v>
-      </c>
       <c r="U41" t="n">
-        <v>2.198068889706438</v>
+        <v>0</v>
       </c>
       <c r="V41" t="n">
-        <v>0.007062670572029382</v>
+        <v>28.24180554491312</v>
       </c>
       <c r="W41" t="n">
-        <v>0.1088380779834294</v>
+        <v>2.198068908667902</v>
       </c>
       <c r="X41" t="n">
+        <v>0.007068164159168635</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>0.1089932301946586</v>
+      </c>
+      <c r="Z41" t="n">
         <v>0.007053333333333333</v>
       </c>
-      <c r="Y41" t="n">
-        <v>24.01327158029936</v>
+      <c r="AA41" t="n">
+        <v>24.01327122841171</v>
       </c>
     </row>
     <row r="42">
@@ -3934,28 +4184,34 @@
         <v>0.03670292593065684</v>
       </c>
       <c r="R42" t="n">
+        <v>0.03606976413308337</v>
+      </c>
+      <c r="S42" t="n">
+        <v>0.1915800770713303</v>
+      </c>
+      <c r="T42" t="n">
         <v>27.80357142857142</v>
       </c>
-      <c r="S42" t="n">
+      <c r="U42" t="n">
         <v>0.05060060245371522</v>
       </c>
-      <c r="T42" t="n">
-        <v>28.47191369338541</v>
-      </c>
-      <c r="U42" t="n">
-        <v>2.203329228300105</v>
-      </c>
       <c r="V42" t="n">
-        <v>0.007575500360812597</v>
+        <v>28.47191433675219</v>
       </c>
       <c r="W42" t="n">
-        <v>0.1171354979034436</v>
+        <v>2.203329247622887</v>
       </c>
       <c r="X42" t="n">
+        <v>0.007575498547917375</v>
+      </c>
+      <c r="Y42" t="n">
+        <v>0.1171354497979989</v>
+      </c>
+      <c r="Z42" t="n">
         <v>0.007626666666666667</v>
       </c>
-      <c r="Y42" t="n">
-        <v>28.24180486772746</v>
+      <c r="AA42" t="n">
+        <v>28.24180554491312</v>
       </c>
     </row>
     <row r="43">
@@ -4017,28 +4273,34 @@
         <v>0.03226430616673658</v>
       </c>
       <c r="R43" t="n">
+        <v>0.03344169305227099</v>
+      </c>
+      <c r="S43" t="n">
+        <v>0.1796226772062386</v>
+      </c>
+      <c r="T43" t="n">
         <v>28.21071428571433</v>
       </c>
-      <c r="S43" t="n">
+      <c r="U43" t="n">
         <v>0.1044036282464569</v>
       </c>
-      <c r="T43" t="n">
-        <v>28.65987999470776</v>
-      </c>
-      <c r="U43" t="n">
-        <v>2.207644899282438</v>
-      </c>
       <c r="V43" t="n">
-        <v>0.007944459054254931</v>
+        <v>28.65988059431129</v>
       </c>
       <c r="W43" t="n">
-        <v>0.1229649217430691</v>
+        <v>2.20764491860522</v>
       </c>
       <c r="X43" t="n">
+        <v>0.007944458816790421</v>
+      </c>
+      <c r="Y43" t="n">
+        <v>0.1229649184265571</v>
+      </c>
+      <c r="Z43" t="n">
         <v>0.008066666666666666</v>
       </c>
-      <c r="Y43" t="n">
-        <v>28.47191369338541</v>
+      <c r="AA43" t="n">
+        <v>28.47191433675219</v>
       </c>
     </row>
     <row r="44">
@@ -4100,28 +4362,34 @@
         <v>0.02491516024776152</v>
       </c>
       <c r="R44" t="n">
+        <v>0.02890464370079389</v>
+      </c>
+      <c r="S44" t="n">
+        <v>0.1578453681542842</v>
+      </c>
+      <c r="T44" t="n">
         <v>28.84999999999995</v>
       </c>
-      <c r="S44" t="n">
+      <c r="U44" t="n">
         <v>0.1491197853115378</v>
       </c>
-      <c r="T44" t="n">
-        <v>28.9256375489027</v>
-      </c>
-      <c r="U44" t="n">
-        <v>2.213775572079771</v>
-      </c>
       <c r="V44" t="n">
-        <v>0.008420554940521486</v>
+        <v>28.92563808749308</v>
       </c>
       <c r="W44" t="n">
-        <v>0.1305037237830004</v>
+        <v>2.213775591402554</v>
       </c>
       <c r="X44" t="n">
+        <v>0.008420554709994834</v>
+      </c>
+      <c r="Y44" t="n">
+        <v>0.1305037205317169</v>
+      </c>
+      <c r="Z44" t="n">
         <v>0.008653333333333332</v>
       </c>
-      <c r="Y44" t="n">
-        <v>28.65987999470776</v>
+      <c r="AA44" t="n">
+        <v>28.65988059431129</v>
       </c>
     </row>
     <row r="45">
@@ -4183,28 +4451,34 @@
         <v>0.01583178431944987</v>
       </c>
       <c r="R45" t="n">
+        <v>0.02290151451210537</v>
+      </c>
+      <c r="S45" t="n">
+        <v>0.1258244186135977</v>
+      </c>
+      <c r="T45" t="n">
         <v>29.8214285714287</v>
       </c>
-      <c r="S45" t="n">
+      <c r="U45" t="n">
         <v>0.1918414613393818</v>
       </c>
-      <c r="T45" t="n">
-        <v>29.46262799265684</v>
-      </c>
-      <c r="U45" t="n">
-        <v>2.226267723460799</v>
-      </c>
       <c r="V45" t="n">
-        <v>0.009253028607806763</v>
+        <v>29.46262840771122</v>
       </c>
       <c r="W45" t="n">
-        <v>0.14371850055597</v>
+        <v>2.226267742783581</v>
       </c>
       <c r="X45" t="n">
+        <v>0.009253028396770656</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>0.1437184974817057</v>
+      </c>
+      <c r="Z45" t="n">
         <v>0.009740000000000002</v>
       </c>
-      <c r="Y45" t="n">
-        <v>28.9256375489027</v>
+      <c r="AA45" t="n">
+        <v>28.92563808749308</v>
       </c>
     </row>
     <row r="46">
@@ -4266,28 +4540,34 @@
         <v>0.003813578138281135</v>
       </c>
       <c r="R46" t="n">
+        <v>0.01083418489561089</v>
+      </c>
+      <c r="S46" t="n">
+        <v>0.0617541750676109</v>
+      </c>
+      <c r="T46" t="n">
         <v>30.18571428571434</v>
       </c>
-      <c r="S46" t="n">
+      <c r="U46" t="n">
         <v>0.2448076315621145</v>
       </c>
-      <c r="T46" t="n">
-        <v>30.73245487163991</v>
-      </c>
-      <c r="U46" t="n">
-        <v>2.256376503569549</v>
-      </c>
       <c r="V46" t="n">
-        <v>0.01074722319542253</v>
+        <v>30.73245500743434</v>
       </c>
       <c r="W46" t="n">
-        <v>0.1673901349917643</v>
+        <v>2.256376522892332</v>
       </c>
       <c r="X46" t="n">
+        <v>0.01074724495172402</v>
+      </c>
+      <c r="Y46" t="n">
+        <v>0.1673908057509535</v>
+      </c>
+      <c r="Z46" t="n">
         <v>0.01196</v>
       </c>
-      <c r="Y46" t="n">
-        <v>29.46262799265684</v>
+      <c r="AA46" t="n">
+        <v>29.46262840771122</v>
       </c>
     </row>
     <row r="47">
@@ -4349,28 +4629,34 @@
         <v>0.002635143243149769</v>
       </c>
       <c r="R47" t="n">
+        <v>0.008945242501938901</v>
+      </c>
+      <c r="S47" t="n">
+        <v>0.05133364630678176</v>
+      </c>
+      <c r="T47" t="n">
         <v>32.48928571428564</v>
       </c>
-      <c r="S47" t="n">
+      <c r="U47" t="n">
         <v>0.2862295508009267</v>
       </c>
-      <c r="T47" t="n">
-        <v>31.15248097080469</v>
-      </c>
-      <c r="U47" t="n">
-        <v>2.266515763708799</v>
-      </c>
       <c r="V47" t="n">
-        <v>0.01113714943474031</v>
+        <v>31.15248101756942</v>
       </c>
       <c r="W47" t="n">
-        <v>0.1734922688738111</v>
+        <v>2.266515783031581</v>
       </c>
       <c r="X47" t="n">
+        <v>0.0111372695428132</v>
+      </c>
+      <c r="Y47" t="n">
+        <v>0.1734960122774931</v>
+      </c>
+      <c r="Z47" t="n">
         <v>0.01262</v>
       </c>
-      <c r="Y47" t="n">
-        <v>30.73245487163991</v>
+      <c r="AA47" t="n">
+        <v>30.73245500743434</v>
       </c>
     </row>
     <row r="48">
@@ -4432,28 +4718,34 @@
         <v>0.003468413842637606</v>
       </c>
       <c r="R48" t="n">
+        <v>0.01023902645998351</v>
+      </c>
+      <c r="S48" t="n">
+        <v>0.05889324106073299</v>
+      </c>
+      <c r="T48" t="n">
         <v>32.9321428571429</v>
       </c>
-      <c r="S48" t="n">
+      <c r="U48" t="n">
         <v>0.2889524121591054</v>
       </c>
-      <c r="T48" t="n">
-        <v>31.55039960390232</v>
-      </c>
-      <c r="U48" t="n">
-        <v>2.276205773398799</v>
-      </c>
       <c r="V48" t="n">
-        <v>0.01147081403029764</v>
+        <v>31.55039956771036</v>
       </c>
       <c r="W48" t="n">
-        <v>0.1786668611418356</v>
+        <v>2.276205792721581</v>
       </c>
       <c r="X48" t="n">
+        <v>0.01147072886081365</v>
+      </c>
+      <c r="Y48" t="n">
+        <v>0.1786641753611795</v>
+      </c>
+      <c r="Z48" t="n">
         <v>0.01322</v>
       </c>
-      <c r="Y48" t="n">
-        <v>31.15248097080469</v>
+      <c r="AA48" t="n">
+        <v>31.15248101756942</v>
       </c>
     </row>
     <row r="49">
@@ -4515,28 +4807,34 @@
         <v>0.004427144891717553</v>
       </c>
       <c r="R49" t="n">
+        <v>0.01153270065092904</v>
+      </c>
+      <c r="S49" t="n">
+        <v>0.06653679351845529</v>
+      </c>
+      <c r="T49" t="n">
         <v>33.08366238246173</v>
       </c>
-      <c r="S49" t="n">
+      <c r="U49" t="n">
         <v>0.2916972101212668</v>
       </c>
-      <c r="T49" t="n">
-        <v>31.95385449152545</v>
-      </c>
-      <c r="U49" t="n">
-        <v>2.286115561086354</v>
-      </c>
       <c r="V49" t="n">
-        <v>0.0117772325789504</v>
+        <v>31.95385437249574</v>
       </c>
       <c r="W49" t="n">
-        <v>0.1833472602095393</v>
+        <v>2.286115580409136</v>
       </c>
       <c r="X49" t="n">
+        <v>0.01177719446570448</v>
+      </c>
+      <c r="Y49" t="n">
+        <v>0.1833460432925698</v>
+      </c>
+      <c r="Z49" t="n">
         <v>0.01380666666666667</v>
       </c>
-      <c r="Y49" t="n">
-        <v>31.55039960390232</v>
+      <c r="AA49" t="n">
+        <v>31.55039956771036</v>
       </c>
     </row>
     <row r="50">
@@ -4598,28 +4896,34 @@
         <v>0.006989072490978496</v>
       </c>
       <c r="R50" t="n">
+        <v>0.01414625769441237</v>
+      </c>
+      <c r="S50" t="n">
+        <v>0.08360067279022637</v>
+      </c>
+      <c r="T50" t="n">
         <v>33.286006759061</v>
       </c>
-      <c r="S50" t="n">
+      <c r="U50" t="n">
         <v>0.2947411967231239</v>
       </c>
-      <c r="T50" t="n">
-        <v>32.83159453267135</v>
-      </c>
-      <c r="U50" t="n">
-        <v>2.307975805168799</v>
-      </c>
       <c r="V50" t="n">
-        <v>0.01235144894981185</v>
+        <v>32.83159423889894</v>
       </c>
       <c r="W50" t="n">
-        <v>0.1918541072094664</v>
+        <v>2.307975824491581</v>
       </c>
       <c r="X50" t="n">
+        <v>0.01235149451992449</v>
+      </c>
+      <c r="Y50" t="n">
+        <v>0.1918556034210608</v>
+      </c>
+      <c r="Z50" t="n">
         <v>0.01502</v>
       </c>
-      <c r="Y50" t="n">
-        <v>31.95385449152545</v>
+      <c r="AA50" t="n">
+        <v>31.95385437249574</v>
       </c>
     </row>
     <row r="51">
@@ -4681,28 +4985,34 @@
         <v>0.01216839656025612</v>
       </c>
       <c r="R51" t="n">
+        <v>0.01855989829652208</v>
+      </c>
+      <c r="S51" t="n">
+        <v>0.1103104553533169</v>
+      </c>
+      <c r="T51" t="n">
         <v>34.92500000000002</v>
       </c>
-      <c r="S51" t="n">
+      <c r="U51" t="n">
         <v>0.3061500936386944</v>
       </c>
-      <c r="T51" t="n">
-        <v>33.75408934841732</v>
-      </c>
-      <c r="U51" t="n">
-        <v>2.331405828598798</v>
-      </c>
       <c r="V51" t="n">
-        <v>0.01284354032424172</v>
+        <v>33.75408893078473</v>
       </c>
       <c r="W51" t="n">
-        <v>0.1986888771392174</v>
+        <v>2.331405847921581</v>
       </c>
       <c r="X51" t="n">
+        <v>0.01284345245977919</v>
+      </c>
+      <c r="Y51" t="n">
+        <v>0.1986859108423037</v>
+      </c>
+      <c r="Z51" t="n">
         <v>0.01622</v>
       </c>
-      <c r="Y51" t="n">
-        <v>32.83159453267135</v>
+      <c r="AA51" t="n">
+        <v>32.83159423889894</v>
       </c>
     </row>
     <row r="52">
@@ -4764,28 +5074,34 @@
         <v>0.01961652719811411</v>
       </c>
       <c r="R52" t="n">
+        <v>0.02311497993131076</v>
+      </c>
+      <c r="S52" t="n">
+        <v>0.1400590132698146</v>
+      </c>
+      <c r="T52" t="n">
         <v>35.32500000000002</v>
       </c>
-      <c r="S52" t="n">
+      <c r="U52" t="n">
         <v>0.3308651428571041</v>
       </c>
-      <c r="T52" t="n">
-        <v>34.61647934287152</v>
-      </c>
-      <c r="U52" t="n">
-        <v>2.353743628714354</v>
-      </c>
       <c r="V52" t="n">
-        <v>0.01322023279290888</v>
+        <v>34.6164789037036</v>
       </c>
       <c r="W52" t="n">
-        <v>0.2034031158610907</v>
+        <v>2.353743648037137</v>
       </c>
       <c r="X52" t="n">
+        <v>0.01322031243075041</v>
+      </c>
+      <c r="Y52" t="n">
+        <v>0.2034058721493541</v>
+      </c>
+      <c r="Z52" t="n">
         <v>0.01728666666666667</v>
       </c>
-      <c r="Y52" t="n">
-        <v>33.75408934841732</v>
+      <c r="AA52" t="n">
+        <v>33.75408893078473</v>
       </c>
     </row>
     <row r="53">
@@ -4847,28 +5163,34 @@
         <v>0.02963924799363945</v>
       </c>
       <c r="R53" t="n">
+        <v>0.0284767157115998</v>
+      </c>
+      <c r="S53" t="n">
+        <v>0.1721605297204892</v>
+      </c>
+      <c r="T53" t="n">
         <v>36.71428571428564</v>
       </c>
-      <c r="S53" t="n">
+      <c r="U53" t="n">
         <v>0.3724108962071924</v>
       </c>
-      <c r="T53" t="n">
-        <v>35.52745852248923</v>
-      </c>
-      <c r="U53" t="n">
-        <v>2.377809652780353</v>
-      </c>
       <c r="V53" t="n">
-        <v>0.01354761888355979</v>
+        <v>35.52745806381636</v>
       </c>
       <c r="W53" t="n">
-        <v>0.2068914320190024</v>
+        <v>2.377809672103136</v>
       </c>
       <c r="X53" t="n">
+        <v>0.01354761894834775</v>
+      </c>
+      <c r="Y53" t="n">
+        <v>0.2068914338797341</v>
+      </c>
+      <c r="Z53" t="n">
         <v>0.01836666666666667</v>
       </c>
-      <c r="Y53" t="n">
-        <v>34.61647934287152</v>
+      <c r="AA53" t="n">
+        <v>34.6164789037036</v>
       </c>
     </row>
     <row r="54">
@@ -4924,34 +5246,40 @@
         <v>0.04417757490269928</v>
       </c>
       <c r="P54" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q54" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R54" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S54" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T54" t="n">
         <v>21.79285714285717</v>
       </c>
-      <c r="S54" t="n">
-        <v>0</v>
-      </c>
-      <c r="T54" t="n">
-        <v>28.31815807173002</v>
-      </c>
       <c r="U54" t="n">
-        <v>2.196892806246272</v>
+        <v>0</v>
       </c>
       <c r="V54" t="n">
-        <v>0.0104122458017144</v>
+        <v>28.31816032897402</v>
       </c>
       <c r="W54" t="n">
-        <v>0.2041952841576134</v>
+        <v>2.196892860793617</v>
       </c>
       <c r="X54" t="n">
+        <v>0.01041304424064643</v>
+      </c>
+      <c r="Y54" t="n">
+        <v>0.2042179130067702</v>
+      </c>
+      <c r="Z54" t="n">
         <v>0.007033333333333333</v>
       </c>
-      <c r="Y54" t="n">
-        <v>25.42114773996207</v>
+      <c r="AA54" t="n">
+        <v>25.42114792085842</v>
       </c>
     </row>
     <row r="55">
@@ -5007,34 +5335,40 @@
         <v>0.02615548495855645</v>
       </c>
       <c r="P55" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q55" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R55" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S55" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T55" t="n">
         <v>22.74159954433088</v>
       </c>
-      <c r="S55" t="n">
-        <v>0</v>
-      </c>
-      <c r="T55" t="n">
-        <v>28.49544506706755</v>
-      </c>
       <c r="U55" t="n">
-        <v>2.2009444491868</v>
+        <v>0</v>
       </c>
       <c r="V55" t="n">
-        <v>0.01098361402771199</v>
+        <v>28.49544748119097</v>
       </c>
       <c r="W55" t="n">
-        <v>0.2161400311342437</v>
+        <v>2.200944508712678</v>
       </c>
       <c r="X55" t="n">
+        <v>0.01098357822667265</v>
+      </c>
+      <c r="Y55" t="n">
+        <v>0.216139031898086</v>
+      </c>
+      <c r="Z55" t="n">
         <v>0.007480000000000001</v>
       </c>
-      <c r="Y55" t="n">
-        <v>28.31815807173002</v>
+      <c r="AA55" t="n">
+        <v>28.31816032897402</v>
       </c>
     </row>
     <row r="56">
@@ -5090,34 +5424,40 @@
         <v>0.02647932083128075</v>
       </c>
       <c r="P56" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q56" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R56" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S56" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T56" t="n">
         <v>22.97108767528296</v>
       </c>
-      <c r="S56" t="n">
-        <v>0</v>
-      </c>
-      <c r="T56" t="n">
-        <v>28.74377626810038</v>
-      </c>
       <c r="U56" t="n">
-        <v>2.206644899331689</v>
+        <v>0</v>
       </c>
       <c r="V56" t="n">
-        <v>0.01171779493992934</v>
+        <v>28.74377861466887</v>
       </c>
       <c r="W56" t="n">
-        <v>0.231737203693045</v>
+        <v>2.206644958857567</v>
       </c>
       <c r="X56" t="n">
+        <v>0.01171774454065133</v>
+      </c>
+      <c r="Y56" t="n">
+        <v>0.2317357767803047</v>
+      </c>
+      <c r="Z56" t="n">
         <v>0.008066666666666666</v>
       </c>
-      <c r="Y56" t="n">
-        <v>28.49544506706755</v>
+      <c r="AA56" t="n">
+        <v>28.49544748119097</v>
       </c>
     </row>
     <row r="57">
@@ -5173,34 +5513,40 @@
         <v>0.02163341820285943</v>
       </c>
       <c r="P57" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q57" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R57" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S57" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T57" t="n">
         <v>24.12500000000008</v>
       </c>
-      <c r="S57" t="n">
-        <v>0</v>
-      </c>
-      <c r="T57" t="n">
-        <v>28.95676810524078</v>
-      </c>
       <c r="U57" t="n">
-        <v>2.211557709800049</v>
+        <v>0</v>
       </c>
       <c r="V57" t="n">
-        <v>0.01228114874974565</v>
+        <v>28.95677039510294</v>
       </c>
       <c r="W57" t="n">
-        <v>0.2438049010993913</v>
+        <v>2.211557769325928</v>
       </c>
       <c r="X57" t="n">
+        <v>0.01228110398018093</v>
+      </c>
+      <c r="Y57" t="n">
+        <v>0.2438036270068062</v>
+      </c>
+      <c r="Z57" t="n">
         <v>0.008539999999999999</v>
       </c>
-      <c r="Y57" t="n">
-        <v>28.74377626810038</v>
+      <c r="AA57" t="n">
+        <v>28.74377861466887</v>
       </c>
     </row>
     <row r="58">
@@ -5256,34 +5602,40 @@
         <v>0.01944191146369945</v>
       </c>
       <c r="P58" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q58" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R58" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S58" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T58" t="n">
         <v>24.57500000000017</v>
       </c>
-      <c r="S58" t="n">
-        <v>0</v>
-      </c>
-      <c r="T58" t="n">
-        <v>29.23616617039069</v>
-      </c>
       <c r="U58" t="n">
-        <v>2.218035494055605</v>
+        <v>0</v>
       </c>
       <c r="V58" t="n">
-        <v>0.01296732616405267</v>
+        <v>29.2361683854742</v>
       </c>
       <c r="W58" t="n">
-        <v>0.2588153203139437</v>
+        <v>2.218035553581483</v>
       </c>
       <c r="X58" t="n">
+        <v>0.01296734667627982</v>
+      </c>
+      <c r="Y58" t="n">
+        <v>0.2588159428505661</v>
+      </c>
+      <c r="Z58" t="n">
         <v>0.009126666666666668</v>
       </c>
-      <c r="Y58" t="n">
-        <v>28.95676810524078</v>
+      <c r="AA58" t="n">
+        <v>28.95677039510294</v>
       </c>
     </row>
     <row r="59">
@@ -5339,34 +5691,40 @@
         <v>0.01658310436687791</v>
       </c>
       <c r="P59" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q59" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R59" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S59" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T59" t="n">
         <v>25.06785714285721</v>
       </c>
-      <c r="S59" t="n">
-        <v>0</v>
-      </c>
-      <c r="T59" t="n">
-        <v>29.78688303409221</v>
-      </c>
       <c r="U59" t="n">
-        <v>2.230915506935605</v>
+        <v>0</v>
       </c>
       <c r="V59" t="n">
-        <v>0.01413302613406024</v>
+        <v>29.78688518662393</v>
       </c>
       <c r="W59" t="n">
-        <v>0.2848787841656656</v>
+        <v>2.230915566461483</v>
       </c>
       <c r="X59" t="n">
+        <v>0.01413308769286362</v>
+      </c>
+      <c r="Y59" t="n">
+        <v>0.2848806420287301</v>
+      </c>
+      <c r="Z59" t="n">
         <v>0.01019333333333333</v>
       </c>
-      <c r="Y59" t="n">
-        <v>29.23616617039069</v>
+      <c r="AA59" t="n">
+        <v>29.2361683854742</v>
       </c>
     </row>
     <row r="60">
@@ -5422,34 +5780,40 @@
         <v>0.01821926693166444</v>
       </c>
       <c r="P60" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q60" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R60" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S60" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T60" t="n">
         <v>25.90000000000013</v>
       </c>
-      <c r="S60" t="n">
-        <v>0</v>
-      </c>
-      <c r="T60" t="n">
-        <v>31.11037299829884</v>
-      </c>
       <c r="U60" t="n">
-        <v>2.262489288509355</v>
+        <v>0</v>
       </c>
       <c r="V60" t="n">
-        <v>0.01625169104512008</v>
+        <v>31.11037508564176</v>
       </c>
       <c r="W60" t="n">
-        <v>0.3347232131708391</v>
+        <v>2.262489348035233</v>
       </c>
       <c r="X60" t="n">
+        <v>0.01625131044668814</v>
+      </c>
+      <c r="Y60" t="n">
+        <v>0.3347113995646889</v>
+      </c>
+      <c r="Z60" t="n">
         <v>0.01242666666666667</v>
       </c>
-      <c r="Y60" t="n">
-        <v>29.78688303409221</v>
+      <c r="AA60" t="n">
+        <v>29.78688518662393</v>
       </c>
     </row>
     <row r="61">
@@ -5505,34 +5869,40 @@
         <v>0.01480594697664882</v>
       </c>
       <c r="P61" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q61" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R61" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S61" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T61" t="n">
         <v>27.37499999999996</v>
       </c>
-      <c r="S61" t="n">
-        <v>0</v>
-      </c>
-      <c r="T61" t="n">
-        <v>31.52104556401108</v>
-      </c>
       <c r="U61" t="n">
-        <v>2.272468965155688</v>
+        <v>0</v>
       </c>
       <c r="V61" t="n">
-        <v>0.01678984232084768</v>
+        <v>31.5210476313021</v>
       </c>
       <c r="W61" t="n">
-        <v>0.3481727318040841</v>
+        <v>2.272469024681567</v>
       </c>
       <c r="X61" t="n">
+        <v>0.01679001717135276</v>
+      </c>
+      <c r="Y61" t="n">
+        <v>0.3481782708526754</v>
+      </c>
+      <c r="Z61" t="n">
         <v>0.01305333333333333</v>
       </c>
-      <c r="Y61" t="n">
-        <v>31.11037299829884</v>
+      <c r="AA61" t="n">
+        <v>31.11037508564176</v>
       </c>
     </row>
     <row r="62">
@@ -5588,34 +5958,40 @@
         <v>0.01899552184075797</v>
       </c>
       <c r="P62" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q62" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R62" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S62" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T62" t="n">
         <v>28.11428571428576</v>
       </c>
-      <c r="S62" t="n">
-        <v>0</v>
-      </c>
-      <c r="T62" t="n">
-        <v>31.94343200681957</v>
-      </c>
       <c r="U62" t="n">
-        <v>2.282825558845605</v>
+        <v>0</v>
       </c>
       <c r="V62" t="n">
-        <v>0.01726821272876278</v>
+        <v>31.94343405366691</v>
       </c>
       <c r="W62" t="n">
-        <v>0.3602759005648064</v>
+        <v>2.282825618371483</v>
       </c>
       <c r="X62" t="n">
+        <v>0.01726817068693205</v>
+      </c>
+      <c r="Y62" t="n">
+        <v>0.3602745856788814</v>
+      </c>
+      <c r="Z62" t="n">
         <v>0.01367333333333333</v>
       </c>
-      <c r="Y62" t="n">
-        <v>31.52104556401108</v>
+      <c r="AA62" t="n">
+        <v>31.5210476313021</v>
       </c>
     </row>
     <row r="63">
@@ -5671,34 +6047,40 @@
         <v>0.02233579751349438</v>
       </c>
       <c r="P63" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q63" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R63" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S63" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T63" t="n">
         <v>28.14285714285706</v>
       </c>
-      <c r="S63" t="n">
-        <v>0</v>
-      </c>
-      <c r="T63" t="n">
-        <v>32.35740187371602</v>
-      </c>
       <c r="U63" t="n">
-        <v>2.293067791310049</v>
+        <v>0</v>
       </c>
       <c r="V63" t="n">
-        <v>0.01769926545816089</v>
+        <v>32.35740390067283</v>
       </c>
       <c r="W63" t="n">
-        <v>0.371479868678853</v>
+        <v>2.293067850835928</v>
       </c>
       <c r="X63" t="n">
+        <v>0.01769926548522211</v>
+      </c>
+      <c r="Y63" t="n">
+        <v>0.3714798980485495</v>
+      </c>
+      <c r="Z63" t="n">
         <v>0.01426</v>
       </c>
-      <c r="Y63" t="n">
-        <v>31.94343200681957</v>
+      <c r="AA63" t="n">
+        <v>31.94343405366691</v>
       </c>
     </row>
     <row r="64">
@@ -5754,34 +6136,40 @@
         <v>0.01014663618242141</v>
       </c>
       <c r="P64" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q64" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R64" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S64" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T64" t="n">
         <v>29.46071428571427</v>
       </c>
-      <c r="S64" t="n">
-        <v>0</v>
-      </c>
-      <c r="T64" t="n">
-        <v>33.2558324964522</v>
-      </c>
       <c r="U64" t="n">
-        <v>2.315615591635606</v>
+        <v>0</v>
       </c>
       <c r="V64" t="n">
-        <v>0.01851302896468444</v>
+        <v>33.25583448054279</v>
       </c>
       <c r="W64" t="n">
-        <v>0.3934451172228779</v>
+        <v>2.315615651161483</v>
       </c>
       <c r="X64" t="n">
+        <v>0.01851307209935324</v>
+      </c>
+      <c r="Y64" t="n">
+        <v>0.3934465808882616</v>
+      </c>
+      <c r="Z64" t="n">
         <v>0.01547333333333333</v>
       </c>
-      <c r="Y64" t="n">
-        <v>32.35740187371602</v>
+      <c r="AA64" t="n">
+        <v>32.35740390067283</v>
       </c>
     </row>
     <row r="65">
@@ -5837,34 +6225,40 @@
         <v>0.00902987934884078</v>
       </c>
       <c r="P65" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q65" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R65" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S65" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T65" t="n">
         <v>30.54107142857147</v>
       </c>
-      <c r="S65" t="n">
-        <v>0</v>
-      </c>
-      <c r="T65" t="n">
-        <v>34.19735342975477</v>
-      </c>
       <c r="U65" t="n">
-        <v>2.339725615745605</v>
+        <v>0</v>
       </c>
       <c r="V65" t="n">
-        <v>0.01919067788683726</v>
+        <v>34.19735536914632</v>
       </c>
       <c r="W65" t="n">
-        <v>0.412573497054656</v>
+        <v>2.339725675271483</v>
       </c>
       <c r="X65" t="n">
+        <v>0.01919069898130528</v>
+      </c>
+      <c r="Y65" t="n">
+        <v>0.4125742480274263</v>
+      </c>
+      <c r="Z65" t="n">
         <v>0.01667333333333334</v>
       </c>
-      <c r="Y65" t="n">
-        <v>33.2558324964522</v>
+      <c r="AA65" t="n">
+        <v>33.25583448054279</v>
       </c>
     </row>
     <row r="66">
@@ -5920,34 +6314,40 @@
         <v>0.01371968923896166</v>
       </c>
       <c r="P66" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q66" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R66" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S66" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T66" t="n">
         <v>30.00357142857132</v>
       </c>
-      <c r="S66" t="n">
-        <v>0</v>
-      </c>
-      <c r="T66" t="n">
-        <v>34.69219227762835</v>
-      </c>
       <c r="U66" t="n">
-        <v>2.3525996008418</v>
+        <v>0</v>
       </c>
       <c r="V66" t="n">
-        <v>0.01948925539598507</v>
+        <v>34.69219417667006</v>
       </c>
       <c r="W66" t="n">
-        <v>0.4213085438452883</v>
+        <v>2.352599660367677</v>
       </c>
       <c r="X66" t="n">
+        <v>0.01948898852875239</v>
+      </c>
+      <c r="Y66" t="n">
+        <v>0.4212993151451641</v>
+      </c>
+      <c r="Z66" t="n">
         <v>0.01728</v>
       </c>
-      <c r="Y66" t="n">
-        <v>34.19735342975477</v>
+      <c r="AA66" t="n">
+        <v>34.19735536914632</v>
       </c>
     </row>
     <row r="67">
@@ -6003,34 +6403,40 @@
         <v>0.0224321685275548</v>
       </c>
       <c r="P67" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="Q67" t="n">
-        <v>0</v>
+        <v>1e-08</v>
       </c>
       <c r="R67" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="S67" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T67" t="n">
         <v>30.12857142857151</v>
       </c>
-      <c r="S67" t="n">
-        <v>0</v>
-      </c>
-      <c r="T67" t="n">
-        <v>35.0418357938299</v>
-      </c>
       <c r="U67" t="n">
-        <v>2.36178186002405</v>
+        <v>0</v>
       </c>
       <c r="V67" t="n">
-        <v>0.01970497486348605</v>
+        <v>35.04183767661643</v>
       </c>
       <c r="W67" t="n">
-        <v>0.4278830064061876</v>
+        <v>2.361781919549927</v>
       </c>
       <c r="X67" t="n">
+        <v>0.01970497329658792</v>
+      </c>
+      <c r="Y67" t="n">
+        <v>0.4278829811081218</v>
+      </c>
+      <c r="Z67" t="n">
         <v>0.0177</v>
       </c>
-      <c r="Y67" t="n">
-        <v>34.69219227762835</v>
+      <c r="AA67" t="n">
+        <v>34.69219417667006</v>
       </c>
     </row>
   </sheetData>

</xml_diff>